<commit_message>
Update 13 May 2026
</commit_message>
<xml_diff>
--- a/WeeklyReports/Component-Oreder-11MAY26.xlsx
+++ b/WeeklyReports/Component-Oreder-11MAY26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\documentsA\WeeklyReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6F09830-49BB-4D6D-9CD6-943AA7B55B00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{062E70AA-4CAC-4935-AC0D-C04D179EF905}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3045" yWindow="3120" windowWidth="28800" windowHeight="11835" xr2:uid="{4C02F06D-BEA5-4673-BADB-5EF96FDAFD89}"/>
   </bookViews>
@@ -55,7 +55,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -68,6 +68,14 @@
       <color theme="1"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -87,16 +95,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -412,7 +425,7 @@
   <dimension ref="B2:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="149.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="149.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
@@ -423,8 +436,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="2" t="s">
         <v>0</v>
       </c>
       <c r="D3">
@@ -448,6 +461,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{13447B5F-C75A-4367-900A-40ADF73AF78E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>